<commit_message>
Fix supplier AP balances: correct X0022+ payments, include X0043, show per-supplier table in dashboard
</commit_message>
<xml_diff>
--- a/Sales_Report.xlsx
+++ b/Sales_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardobazua/bza-reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05A5DB15-2C95-5642-98D8-7571C5D0827D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1C2C7B-5645-834D-B675-B9049519E079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="820" windowWidth="30240" windowHeight="17480" xr2:uid="{A69E99B4-FD75-534F-A443-AF5D6F49D11E}"/>
+    <workbookView xWindow="0" yWindow="820" windowWidth="30240" windowHeight="17480" xr2:uid="{A69E99B4-FD75-534F-A443-AF5D6F49D11E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -7058,12 +7058,11 @@
       </c>
       <c r="U67" s="28"/>
       <c r="V67" s="42">
-        <f>SUM(R67:T67)</f>
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="W67" s="28">
         <f>O67*V67</f>
-        <v>339410.24</v>
+        <v>323053.12</v>
       </c>
       <c r="X67" s="28">
         <v>705</v>
@@ -7084,7 +7083,7 @@
       </c>
       <c r="AD67" s="28">
         <f>AC67-W67</f>
-        <v>20957.560000000056</v>
+        <v>37314.680000000051</v>
       </c>
       <c r="AE67" t="s">
         <v>82</v>
@@ -7142,12 +7141,11 @@
       </c>
       <c r="U68" s="28"/>
       <c r="V68" s="42">
-        <f>SUM(R68:T68)</f>
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="W68" s="28">
         <f>O68*V68</f>
-        <v>338104.81599999999</v>
+        <v>321810.60800000001</v>
       </c>
       <c r="X68" s="28">
         <v>705</v>
@@ -7168,7 +7166,7 @@
       </c>
       <c r="AD68" s="28">
         <f>AC68-W68</f>
-        <v>20876.954000000027</v>
+        <v>37171.162000000011</v>
       </c>
       <c r="AE68" s="17"/>
     </row>
@@ -7224,12 +7222,11 @@
       </c>
       <c r="U69" s="28"/>
       <c r="V69" s="42">
-        <f>SUM(R69:T69)</f>
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="W69" s="28">
         <f>O69*V69</f>
-        <v>322061.91200000001</v>
+        <v>306540.85600000003</v>
       </c>
       <c r="X69" s="28">
         <v>705</v>
@@ -7250,7 +7247,7 @@
       </c>
       <c r="AD69" s="28">
         <f t="shared" ref="AD69:AD73" si="31">AC69-W69</f>
-        <v>19886.353000000003</v>
+        <v>35407.408999999985</v>
       </c>
     </row>
     <row r="70" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -7305,12 +7302,11 @@
       </c>
       <c r="U70" s="28"/>
       <c r="V70" s="42">
-        <f>SUM(R70:T70)</f>
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="W70" s="28">
         <f>O70*V70</f>
-        <v>338892.32</v>
+        <v>322560.15999999997</v>
       </c>
       <c r="X70" s="28">
         <v>705</v>
@@ -7331,7 +7327,7 @@
       </c>
       <c r="AD70" s="28">
         <f t="shared" si="31"/>
-        <v>20925.580000000016</v>
+        <v>37257.740000000049</v>
       </c>
     </row>
     <row r="71" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -7386,12 +7382,11 @@
       </c>
       <c r="U71" s="28"/>
       <c r="V71" s="42">
-        <f>SUM(R71:T71)</f>
-        <v>664</v>
+        <v>634</v>
       </c>
       <c r="W71" s="28">
         <f>O71*V71</f>
-        <v>321416.50399999996</v>
+        <v>306894.674</v>
       </c>
       <c r="X71" s="28">
         <v>705</v>
@@ -7412,7 +7407,7 @@
       </c>
       <c r="AD71" s="28">
         <f t="shared" si="31"/>
-        <v>19846.501000000047</v>
+        <v>34368.331000000006</v>
       </c>
     </row>
     <row r="72" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -7467,12 +7462,11 @@
       </c>
       <c r="U72" s="28"/>
       <c r="V72" s="42">
-        <f>SUM(R72:T72)</f>
-        <v>664</v>
+        <v>634</v>
       </c>
       <c r="W72" s="28">
         <f>O72*V72</f>
-        <v>321783.696</v>
+        <v>307245.27600000001</v>
       </c>
       <c r="X72" s="28">
         <v>705</v>
@@ -7493,7 +7487,7 @@
       </c>
       <c r="AD72" s="28">
         <f t="shared" si="31"/>
-        <v>19869.173999999999</v>
+        <v>34407.593999999983</v>
       </c>
     </row>
     <row r="73" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -7548,12 +7542,11 @@
       </c>
       <c r="U73" s="28"/>
       <c r="V73" s="42">
-        <f>SUM(R73:T73)</f>
-        <v>664</v>
+        <v>634</v>
       </c>
       <c r="W73" s="28">
         <f>O73*V73</f>
-        <v>321291.67200000002</v>
+        <v>306775.48200000002</v>
       </c>
       <c r="X73" s="28">
         <v>705</v>
@@ -7574,7 +7567,7 @@
       </c>
       <c r="AD73" s="28">
         <f t="shared" si="31"/>
-        <v>19838.792999999947</v>
+        <v>34354.982999999949</v>
       </c>
       <c r="AE73" t="s">
         <v>130</v>
@@ -7632,12 +7625,11 @@
       </c>
       <c r="U74" s="28"/>
       <c r="V74" s="42">
-        <f>SUM(R74:T74)</f>
-        <v>664</v>
+        <v>634</v>
       </c>
       <c r="W74" s="28">
         <f>O74*V74</f>
-        <v>320101.78399999999</v>
+        <v>305639.35399999999</v>
       </c>
       <c r="X74" s="28">
         <v>705</v>
@@ -7658,7 +7650,7 @@
       </c>
       <c r="AD74" s="28">
         <f t="shared" ref="AD74" si="32">AC74-W74</f>
-        <v>19765.321000000054</v>
+        <v>34227.751000000047</v>
       </c>
       <c r="AE74" t="s">
         <v>131</v>
@@ -7716,12 +7708,11 @@
       </c>
       <c r="U75" s="28"/>
       <c r="V75" s="42">
-        <f>SUM(R75:T75)</f>
-        <v>664</v>
+        <v>634</v>
       </c>
       <c r="W75" s="28">
         <f>O75*V75</f>
-        <v>198109.712</v>
+        <v>189158.97200000001</v>
       </c>
       <c r="X75" s="28">
         <v>705</v>
@@ -7742,7 +7733,7 @@
       </c>
       <c r="AD75" s="28">
         <f t="shared" ref="AD75" si="33">AC75-W75</f>
-        <v>12232.678000000014</v>
+        <v>21183.418000000005</v>
       </c>
       <c r="AE75" t="s">
         <v>132</v>
@@ -7781,7 +7772,7 @@
       <c r="V76" s="24"/>
       <c r="W76" s="25">
         <f>+SUM(W67:W75)</f>
-        <v>2821172.656</v>
+        <v>2689678.5019999999</v>
       </c>
       <c r="X76" s="24"/>
       <c r="Y76" s="24"/>
@@ -7794,7 +7785,7 @@
       </c>
       <c r="AD76" s="25">
         <f>+SUM(AD67:AD75)</f>
-        <v>174198.91400000016</v>
+        <v>305693.06800000009</v>
       </c>
     </row>
     <row r="77" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -8504,8 +8495,7 @@
         <v>16</v>
       </c>
       <c r="R84" s="28">
-        <f>K84+30</f>
-        <v>30</v>
+        <v>668</v>
       </c>
       <c r="S84" s="28">
         <v>0</v>
@@ -8516,11 +8506,11 @@
       <c r="U84" s="28"/>
       <c r="V84" s="28">
         <f>R84+T84</f>
-        <v>10</v>
+        <v>648</v>
       </c>
       <c r="W84" s="28">
         <f>O84*V84</f>
-        <v>4982.58</v>
+        <v>322871.18400000001</v>
       </c>
       <c r="X84" s="28">
         <v>740</v>
@@ -8541,7 +8531,7 @@
       </c>
       <c r="AD84" s="28">
         <f>AC84-W84</f>
-        <v>363728.33999999997</v>
+        <v>45839.735999999975</v>
       </c>
       <c r="AE84" s="38" t="s">
         <v>134</v>
@@ -8594,8 +8584,7 @@
         <v>16</v>
       </c>
       <c r="R85" s="28">
-        <f>K85+30</f>
-        <v>30</v>
+        <v>668</v>
       </c>
       <c r="S85" s="28">
         <v>0</v>
@@ -8606,11 +8595,11 @@
       <c r="U85" s="28"/>
       <c r="V85" s="28">
         <f>R85+T85</f>
-        <v>10</v>
+        <v>648</v>
       </c>
       <c r="W85" s="28">
         <f>O85*V85</f>
-        <v>4994.8</v>
+        <v>323663.04000000004</v>
       </c>
       <c r="X85" s="28">
         <v>740</v>
@@ -8631,7 +8620,7 @@
       </c>
       <c r="AD85" s="28">
         <f t="shared" ref="AD85:AD86" si="38">AC85-W85</f>
-        <v>364620.4</v>
+        <v>45952.159999999974</v>
       </c>
       <c r="AE85" s="38" t="s">
         <v>135</v>
@@ -8684,8 +8673,7 @@
         <v>16</v>
       </c>
       <c r="R86" s="28">
-        <f>K86+30</f>
-        <v>30</v>
+        <v>668</v>
       </c>
       <c r="S86" s="28">
         <v>0</v>
@@ -8696,11 +8684,11 @@
       <c r="U86" s="28"/>
       <c r="V86" s="28">
         <f>R86+T86</f>
-        <v>10</v>
+        <v>648</v>
       </c>
       <c r="W86" s="28">
         <f>O86*V86</f>
-        <v>4984.92</v>
+        <v>323022.81599999999</v>
       </c>
       <c r="X86" s="28">
         <v>740</v>
@@ -8721,7 +8709,7 @@
       </c>
       <c r="AD86" s="28">
         <f t="shared" si="38"/>
-        <v>363899.16000000003</v>
+        <v>45861.264000000025</v>
       </c>
       <c r="AE86" s="38" t="s">
         <v>135</v>
@@ -8760,7 +8748,7 @@
       <c r="V87" s="24"/>
       <c r="W87" s="25">
         <f>+SUM(W84:W86)</f>
-        <v>14962.300000000001</v>
+        <v>969557.04</v>
       </c>
       <c r="X87" s="24"/>
       <c r="Y87" s="24"/>
@@ -8773,7 +8761,7 @@
       </c>
       <c r="AD87" s="25">
         <f>+SUM(AD84:AD86)</f>
-        <v>1092247.8999999999</v>
+        <v>137653.15999999997</v>
       </c>
     </row>
     <row r="88" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -8826,8 +8814,7 @@
         <v>16</v>
       </c>
       <c r="R88" s="28">
-        <f>K88+30</f>
-        <v>1032.0709999999999</v>
+        <v>675</v>
       </c>
       <c r="S88" s="28">
         <v>0</v>
@@ -8838,11 +8825,11 @@
       <c r="U88" s="28"/>
       <c r="V88" s="28">
         <f>R88+T88</f>
-        <v>1012.0709999999999</v>
+        <v>655</v>
       </c>
       <c r="W88" s="28">
         <f>O88*V88</f>
-        <v>505140.82923599996</v>
+        <v>326920.98</v>
       </c>
       <c r="X88" s="28">
         <v>740</v>
@@ -8863,7 +8850,7 @@
       </c>
       <c r="AD88" s="28">
         <f t="shared" ref="AD88:AD90" si="39">AC88-W88</f>
-        <v>-135794.98923599999</v>
+        <v>42424.859999999986</v>
       </c>
       <c r="AE88" s="38" t="s">
         <v>175</v>
@@ -8916,8 +8903,7 @@
         <v>16</v>
       </c>
       <c r="R89" s="28">
-        <f>K89+30</f>
-        <v>30</v>
+        <v>675</v>
       </c>
       <c r="S89" s="28">
         <v>0</v>
@@ -8928,11 +8914,11 @@
       <c r="U89" s="28"/>
       <c r="V89" s="28">
         <f>R89+T89</f>
-        <v>10</v>
+        <v>655</v>
       </c>
       <c r="W89" s="28">
         <f>O89*V89</f>
-        <v>4982.7</v>
+        <v>326366.84999999998</v>
       </c>
       <c r="X89" s="28">
         <v>740</v>
@@ -8953,7 +8939,7 @@
       </c>
       <c r="AD89" s="28">
         <f t="shared" si="39"/>
-        <v>363737.1</v>
+        <v>42352.950000000012</v>
       </c>
       <c r="AE89" s="38" t="s">
         <v>185</v>
@@ -9006,8 +8992,7 @@
         <v>16</v>
       </c>
       <c r="R90" s="28">
-        <f>K90+30</f>
-        <v>30</v>
+        <v>675</v>
       </c>
       <c r="S90" s="28">
         <v>0</v>
@@ -9018,11 +9003,11 @@
       <c r="U90" s="28"/>
       <c r="V90" s="28">
         <f>R90+T90</f>
-        <v>10</v>
+        <v>655</v>
       </c>
       <c r="W90" s="28">
         <f>O90*V90</f>
-        <v>4996.18</v>
+        <v>327249.78999999998</v>
       </c>
       <c r="X90" s="28">
         <v>740</v>
@@ -9043,7 +9028,7 @@
       </c>
       <c r="AD90" s="28">
         <f t="shared" si="39"/>
-        <v>364721.14</v>
+        <v>42467.530000000028</v>
       </c>
       <c r="AE90" s="38" t="s">
         <v>196</v>
@@ -9079,7 +9064,7 @@
       <c r="V91" s="24"/>
       <c r="W91" s="25">
         <f>+SUM(W88:W90)</f>
-        <v>515119.70923599997</v>
+        <v>980537.61999999988</v>
       </c>
       <c r="X91" s="24"/>
       <c r="Y91" s="24"/>
@@ -9092,7 +9077,7 @@
       </c>
       <c r="AD91" s="25">
         <f>+SUM(AD88:AD90)</f>
-        <v>592663.250764</v>
+        <v>127245.34000000003</v>
       </c>
     </row>
     <row r="92" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -9801,11 +9786,10 @@
         <v>16</v>
       </c>
       <c r="R99" s="42">
-        <f>K99</f>
-        <v>0</v>
+        <v>616</v>
       </c>
       <c r="S99" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T99" s="28">
         <v>-30</v>
@@ -9813,11 +9797,11 @@
       <c r="U99" s="28"/>
       <c r="V99" s="28">
         <f>R99+T99</f>
-        <v>-30</v>
+        <v>586</v>
       </c>
       <c r="W99" s="28">
         <f>O99*V99</f>
-        <v>-15060.480000000001</v>
+        <v>294181.37599999999</v>
       </c>
       <c r="X99" s="28">
         <v>710</v>
@@ -9838,7 +9822,7 @@
       </c>
       <c r="AD99" s="28">
         <f t="shared" ref="AD99:AD100" si="42">AC99-W99</f>
-        <v>371491.83999999997</v>
+        <v>62249.983999999997</v>
       </c>
       <c r="AE99" s="38" t="s">
         <v>215</v>
@@ -9886,8 +9870,7 @@
         <v>16</v>
       </c>
       <c r="R100" s="42">
-        <f>K100</f>
-        <v>0</v>
+        <v>616</v>
       </c>
       <c r="S100" s="28">
         <v>0</v>
@@ -9898,11 +9881,11 @@
       <c r="U100" s="28"/>
       <c r="V100" s="28">
         <f>R100+T100</f>
-        <v>-30</v>
+        <v>586</v>
       </c>
       <c r="W100" s="28">
         <f>O100*V100</f>
-        <v>-15001.65</v>
+        <v>293032.23</v>
       </c>
       <c r="X100" s="28">
         <v>710</v>
@@ -9923,7 +9906,7 @@
       </c>
       <c r="AD100" s="28">
         <f t="shared" si="42"/>
-        <v>370040.7</v>
+        <v>62006.820000000007</v>
       </c>
       <c r="AE100" s="38" t="s">
         <v>215</v>
@@ -9960,7 +9943,7 @@
       <c r="V101" s="24"/>
       <c r="W101" s="25">
         <f>+SUM(W99:W100)</f>
-        <v>-30062.13</v>
+        <v>587213.60599999991</v>
       </c>
       <c r="X101" s="24"/>
       <c r="Y101" s="24"/>
@@ -9973,7 +9956,7 @@
       </c>
       <c r="AD101" s="25">
         <f>+SUM(AD99:AD100)</f>
-        <v>741532.54</v>
+        <v>124256.804</v>
       </c>
     </row>
     <row r="102" spans="1:44" ht="32" x14ac:dyDescent="0.2">
@@ -18124,7 +18107,7 @@
       </c>
       <c r="AD202" s="17">
         <f>SUM(AD122,AD101,AD91,AD87,AD76,AD66,AD149,)</f>
-        <v>3134788.9567640005</v>
+        <v>1228994.7240000002</v>
       </c>
     </row>
     <row r="203" spans="1:31" x14ac:dyDescent="0.2">
@@ -18624,7 +18607,7 @@
       <c r="Y241" s="68"/>
       <c r="Z241" s="69">
         <f>X84-R84</f>
-        <v>710</v>
+        <v>72</v>
       </c>
       <c r="AA241" s="69"/>
       <c r="AB241" s="70">
@@ -18693,7 +18676,7 @@
       </c>
       <c r="Z243" s="69">
         <f>Z241*Z242</f>
-        <v>1062323.3</v>
+        <v>107728.56</v>
       </c>
       <c r="AA243" s="69"/>
       <c r="AB243" s="70">
@@ -18760,7 +18743,7 @@
       </c>
       <c r="Z245" s="92">
         <f>Z243*Z244</f>
-        <v>382436.38799999998</v>
+        <v>38782.281599999995</v>
       </c>
       <c r="AA245" s="92"/>
       <c r="AB245" s="93">
@@ -18862,7 +18845,7 @@
       <c r="AA249" s="95"/>
       <c r="AB249" s="93">
         <f>AB245+Z245</f>
-        <v>421238.73167999997</v>
+        <v>77584.625279999993</v>
       </c>
       <c r="AC249" s="68" t="s">
         <v>308</v>
@@ -18895,7 +18878,7 @@
       </c>
       <c r="AD250" s="70">
         <f>AB260</f>
-        <v>-332197.73167999997</v>
+        <v>11456.374720000007</v>
       </c>
       <c r="AF250" s="80">
         <v>325000</v>
@@ -18952,7 +18935,7 @@
       </c>
       <c r="AD252" s="100">
         <f>AD249-AD250</f>
-        <v>410896.92343999993</v>
+        <v>67242.81703999998</v>
       </c>
       <c r="AF252" s="80">
         <v>514200</v>
@@ -19013,7 +18996,7 @@
       </c>
       <c r="AD254" s="100">
         <f>AD252-AD253</f>
-        <v>360896.92343999993</v>
+        <v>17242.81703999998</v>
       </c>
       <c r="AF254" s="80">
         <v>632000</v>
@@ -19114,7 +19097,7 @@
       <c r="AA258" s="95"/>
       <c r="AB258" s="93">
         <f>AB249-AB251+AB252-AB253-AB254+AB255+AB256-AB257</f>
-        <v>397197.73167999997</v>
+        <v>53543.625279999993</v>
       </c>
       <c r="AC258" s="68"/>
       <c r="AD258" s="72"/>
@@ -19163,7 +19146,7 @@
       <c r="AA260" s="75"/>
       <c r="AB260" s="102">
         <f>AB259-AB258</f>
-        <v>-332197.73167999997</v>
+        <v>11456.374720000007</v>
       </c>
       <c r="AC260" s="68"/>
       <c r="AD260" s="72"/>
@@ -19391,7 +19374,7 @@
       </c>
       <c r="AE270" s="53">
         <f>SUM(W66,W76,W87,W91,W101,W122)</f>
-        <v>6665813.6082359999</v>
+        <v>8571607.8409999982</v>
       </c>
       <c r="AF270" s="86">
         <f>SUMIF(AJ220:AJ265,"Arauco",AF220:AF265)</f>
@@ -19402,7 +19385,7 @@
       </c>
       <c r="AH270" s="87">
         <f>AE270-AF270</f>
-        <v>-1923415.3917640001</v>
+        <v>-17621.159000001848</v>
       </c>
     </row>
     <row r="271" spans="18:36" x14ac:dyDescent="0.2">
@@ -19451,7 +19434,7 @@
       </c>
       <c r="AE272" s="53">
         <f>SUM(AE270:AE271)</f>
-        <v>11061999.943236001</v>
+        <v>12967794.175999999</v>
       </c>
       <c r="AF272" s="86">
         <f>SUM(AF225:AF265)</f>
@@ -19462,7 +19445,7 @@
       </c>
       <c r="AH272" s="87">
         <f>SUM(AH270:AH271)</f>
-        <v>-1853230.0567640001</v>
+        <v>52564.175999998115</v>
       </c>
     </row>
     <row r="273" spans="24:40" x14ac:dyDescent="0.2">
@@ -20016,7 +19999,7 @@
       </c>
       <c r="AN305" s="17">
         <f>W76</f>
-        <v>2821172.656</v>
+        <v>2689678.5019999999</v>
       </c>
     </row>
     <row r="306" spans="32:40" x14ac:dyDescent="0.2">
@@ -20025,7 +20008,7 @@
       </c>
       <c r="AN306" s="45">
         <f>AN304-AN305</f>
-        <v>-103172.65599999996</v>
+        <v>28321.498000000138</v>
       </c>
     </row>
     <row r="307" spans="32:40" x14ac:dyDescent="0.2">
@@ -20096,7 +20079,7 @@
       </c>
       <c r="AN313" s="17">
         <f>W67+W68+W69+W70+W71+W72+W73+(O74*668)+(O75*668)</f>
-        <v>2824294.412</v>
+        <v>2716213.4279999998</v>
       </c>
     </row>
     <row r="314" spans="32:40" x14ac:dyDescent="0.2">
@@ -20105,7 +20088,7 @@
       </c>
       <c r="AN314" s="45">
         <f>AN312-AN313</f>
-        <v>-106294.41200000001</v>
+        <v>1786.5720000001602</v>
       </c>
     </row>
     <row r="316" spans="32:40" x14ac:dyDescent="0.2">
@@ -20131,11 +20114,11 @@
       </c>
       <c r="AG318" s="17">
         <f>X67-V67</f>
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="AH318" s="17">
         <f>AF318*AG318</f>
-        <v>457.56000000000103</v>
+        <v>814.68000000000188</v>
       </c>
     </row>
     <row r="319" spans="32:40" x14ac:dyDescent="0.2">
@@ -20145,11 +20128,11 @@
       </c>
       <c r="AG319" s="17">
         <f>X68-V68</f>
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="AH319" s="17">
         <f t="shared" ref="AH319:AH326" si="92">AF319*AG319</f>
-        <v>376.95400000000069</v>
+        <v>671.16200000000117</v>
       </c>
     </row>
     <row r="320" spans="32:40" x14ac:dyDescent="0.2">
@@ -20159,11 +20142,11 @@
       </c>
       <c r="AG320" s="17">
         <f>X69-V69</f>
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="AH320" s="17">
         <f t="shared" si="92"/>
-        <v>-613.64699999999937</v>
+        <v>-1092.590999999999</v>
       </c>
     </row>
     <row r="321" spans="32:38" x14ac:dyDescent="0.2">
@@ -20173,11 +20156,11 @@
       </c>
       <c r="AG321" s="17">
         <f>X70-V70</f>
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="AH321" s="17">
         <f t="shared" si="92"/>
-        <v>425.57999999999981</v>
+        <v>757.73999999999967</v>
       </c>
     </row>
     <row r="322" spans="32:38" x14ac:dyDescent="0.2">
@@ -20187,11 +20170,11 @@
       </c>
       <c r="AG322" s="17">
         <f>X71-V71</f>
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="AH322" s="17">
         <f t="shared" si="92"/>
-        <v>-653.49900000000093</v>
+        <v>-1131.6690000000015</v>
       </c>
     </row>
     <row r="323" spans="32:38" x14ac:dyDescent="0.2">
@@ -20201,11 +20184,11 @@
       </c>
       <c r="AG323" s="17">
         <f>X72-V72</f>
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="AH323" s="17">
         <f t="shared" si="92"/>
-        <v>-630.82600000000093</v>
+        <v>-1092.4060000000018</v>
       </c>
     </row>
     <row r="324" spans="32:38" x14ac:dyDescent="0.2">
@@ -20215,11 +20198,11 @@
       </c>
       <c r="AG324" s="17">
         <f>X73-V73</f>
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="AH324" s="17">
         <f t="shared" si="92"/>
-        <v>-661.20700000000033</v>
+        <v>-1145.0170000000007</v>
       </c>
     </row>
     <row r="325" spans="32:38" x14ac:dyDescent="0.2">
@@ -20229,11 +20212,11 @@
       </c>
       <c r="AG325" s="17">
         <f>X74-V74</f>
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="AH325" s="17">
         <f t="shared" si="92"/>
-        <v>-734.67899999999929</v>
+        <v>-1272.2489999999989</v>
       </c>
     </row>
     <row r="326" spans="32:38" x14ac:dyDescent="0.2">
@@ -20243,11 +20226,11 @@
       </c>
       <c r="AG326" s="17">
         <f>X75-V75</f>
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="AH326" s="17">
         <f t="shared" si="92"/>
-        <v>-67.321999999999832</v>
+        <v>-116.58199999999971</v>
       </c>
     </row>
     <row r="327" spans="32:38" x14ac:dyDescent="0.2">
@@ -20265,7 +20248,7 @@
       </c>
       <c r="AH328" s="47">
         <f>SUM(AH318:AH326)</f>
-        <v>-2101.0859999999989</v>
+        <v>-3606.9319999999993</v>
       </c>
     </row>
     <row r="329" spans="32:38" x14ac:dyDescent="0.2">

</xml_diff>